<commit_message>
Update Master Excel with expanded candidate URLs and new venue targets
</commit_message>
<xml_diff>
--- a/South_Bend_Master_Event_Sources.xlsx
+++ b/South_Bend_Master_Event_Sources.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -593,6 +593,21 @@
           <t>Recommended Priority</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Alternate URL Candidate 1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Alternate URL Candidate 2</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Audit Status</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -625,6 +640,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
@@ -657,6 +677,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -689,6 +714,11 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -721,6 +751,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -753,6 +788,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -785,6 +825,16 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://palaisroyale.org/contact</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Discovered 1 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -817,6 +867,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.pigeonhenpottery.com/event-calendar</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Discovered 1 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -849,6 +909,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -881,6 +946,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://sbct.org/shows</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://ci.ovationtix.com/35243</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -913,6 +993,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -945,6 +1030,21 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://southbendart.org/all-events/</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://southbendart.org</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
@@ -977,6 +1077,21 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://southbendsymphony.org/calendar</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://southbendsymphony.org/events</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1009,6 +1124,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://sjcpl.org/special-events/</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://sjcpl.org/programs-events/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
@@ -1041,6 +1171,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1073,6 +1208,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
@@ -1105,6 +1245,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://wellfieldgardens.org/calendar</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.wellfieldgardens.org/calendar</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -1137,6 +1292,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
@@ -1169,6 +1329,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>http://chicoryeventcenter.com</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Discovered 1 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1201,6 +1371,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
@@ -1233,6 +1408,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -1265,6 +1445,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -1297,6 +1482,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -1329,6 +1519,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.journeyman.com/calendar</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.journeyman.com/community/calendar</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="7" t="inlineStr">
@@ -1361,6 +1566,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -1393,6 +1603,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.sunkingbrewing.com/private-events</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Discovered 1 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
@@ -1425,6 +1645,11 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -1457,6 +1682,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.wvpe.org/schedule</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.wvpe.org/all-shows</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
@@ -1489,6 +1729,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://barlouie.com/bar-louie-events/</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://barlouie.com/group-events/</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -1521,6 +1776,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -1553,6 +1813,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.corbysirishpub.com/calendar--special-events.html</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Discovered 1 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
@@ -1585,6 +1855,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
@@ -1617,6 +1892,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://fourwindscasino.com/event-calendar</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://reservations2.fourwindscasino.com/ReservationCalendar.action</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -1649,6 +1939,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="7" t="inlineStr">
@@ -1681,6 +1976,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -1713,6 +2013,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
@@ -1745,6 +2050,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -1777,6 +2087,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
@@ -1809,6 +2124,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
@@ -1841,6 +2161,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
@@ -1873,6 +2198,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://thegeneraldeli.com/general-events</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Discovered 1 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -1905,6 +2240,16 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.kirkwoodcollection.com/hideaway/events-room-blocks/</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Discovered 1 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
@@ -1937,6 +2282,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -1969,6 +2319,11 @@
           <t>Disabled - Domain Dead</t>
         </is>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
@@ -2001,6 +2356,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://sbparksandrec.org/calendar</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://sbparksandrec.org/events</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -2033,6 +2403,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://mishawaka.in.gov/government/departments/police-department/</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://mishawaka.in.gov/government/departments/fire-ems/fire-prevention-bureau/</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
@@ -2065,6 +2450,21 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.potawatomizoo.org/events</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://potawatomizoo.org/events/category/education-events/list/</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
@@ -2097,6 +2497,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.milb.com/schedule</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://www.milb.com/milb/schedule</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
@@ -2129,6 +2544,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://sbvpa.org/shows</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://sbvpa.org/things-to-do</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
@@ -2161,6 +2591,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.sjcparks.org/calendar</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://www.sjcparks.org/518/Programs-Events</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
@@ -2193,6 +2638,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
@@ -2225,6 +2675,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.visitelkhartcounty.com/things-to-do</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://www.visitelkhartcounty.com/events/this-weekend/</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
@@ -2257,6 +2722,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>http://micommunityfinancials.michigan.gov/#!/dashboard/CITY/2657760?lat=41.83453900000001&amp;lng=-86.24785099999997&amp;zoom=10&amp;showSidebar=yes</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://www.nilesmi.org/document_center/department/Clerk/SPECIAL EVENT APPLICATION - fillable.pdf</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -2289,6 +2769,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://southbendin.gov/things-to-do</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://sbvpa.org/things-to-do/</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
@@ -2321,6 +2816,21 @@
           <t>High (Top Target)</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.downtownsouthbend.com/events</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.downtownsouthbend.com/schedule</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -2353,6 +2863,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/things-to-do</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
@@ -2385,6 +2910,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
@@ -2417,6 +2947,21 @@
           <t>High (Top Target)</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.visitsouthbend.com/things-to-do</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.visitsouthbend.com/events/this-weekend/</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
@@ -2449,6 +2994,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://mishawaka.in.gov/events</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://mishawaka.in.gov/government/departments/police-department/</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -2481,6 +3041,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.elkhartindiana.org/things-to-do</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.visitelkhartcounty.com/events/</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="7" t="inlineStr">
@@ -2513,6 +3088,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://myepl.org/calendar</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://myepl.org/community/calendar</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -2545,6 +3135,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.fernwoodbotanical.org/events</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.fernwoodbotanical.org/list-of-events-programs</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="7" t="inlineStr">
@@ -2577,6 +3182,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://downtowngoshen.org/event-calendar</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://downtowngoshen.org/event-calendar/</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -2609,6 +3229,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="7" t="inlineStr">
@@ -2641,6 +3266,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
@@ -2673,6 +3303,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="7" t="inlineStr">
@@ -2705,6 +3340,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://mishawaka.in.gov/events</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://mishawaka.in.gov/things-to-do</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
@@ -2737,6 +3387,11 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="7" t="inlineStr">
@@ -2769,6 +3424,11 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
@@ -2801,6 +3461,21 @@
           <t>High (Top Target)</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/calendar</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/events</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="7" t="inlineStr">
@@ -2833,6 +3508,11 @@
           <t>High</t>
         </is>
       </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
@@ -2865,6 +3545,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/find/?source=EVENTS&amp;eventType=inPerson&amp;sortField=DATETIME&amp;location=us--mi--Saint+Joseph</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/books-banter-a-book-club-for-women/events/316306457/?eventOrigin=home_logged_out_near_location</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="7" t="inlineStr">
@@ -2897,6 +3592,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://promotix.com/event-creators</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://www.promotix.com/event-discovery/l/new</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
@@ -2929,6 +3639,11 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="7" t="inlineStr">
@@ -2961,6 +3676,21 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.hcc-nd.edu/calendar</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.hcc-nd.edu/community/calendar</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
@@ -2993,6 +3723,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://events.iu.edu/events</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://events.iu.edu/event-calendar</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="7" t="inlineStr">
@@ -3025,6 +3770,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://fightingirish.com/sports/baseball/schedule/</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://fightingirish.com/sports/mbball/schedule/</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
@@ -3057,6 +3817,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://performingarts.nd.edu/calendar</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://dpactickets.nd.edu/events</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="7" t="inlineStr">
@@ -3089,6 +3864,21 @@
           <t>High (Top Target)</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://events.nd.edu/events</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://events.nd.edu/submit-an-event</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
@@ -3121,6 +3911,21 @@
           <t>High</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://sao.nd.edu/events/2026/10/31/halloweenfest/</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://sao.nd.edu/events/calendar/featured/</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Discovered 4 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="7" t="inlineStr">
@@ -3153,6 +3958,21 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.saintmarys.edu/academics/resources/academic-calendar</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.saintmarys.edu/spiritual-life/calendar</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
@@ -3185,6 +4005,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://performingarts.nd.edu/calendar</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://performingarts.nd.edu/events</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="7" t="inlineStr">
@@ -3217,6 +4052,11 @@
           <t>Low</t>
         </is>
       </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -3249,6 +4089,21 @@
           <t>High (Top Target)</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://www.langlabsb.com/events</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://www.langlabsb.com/schedule</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="7" t="inlineStr">
@@ -3281,6 +4136,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://merrimansplayhouse.org/events</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://merrimansplayhouse.org/schedule</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="4" t="inlineStr">
@@ -3313,6 +4183,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://morriscenter.org/events</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://morriscenter.org/upcoming-events</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Discovered 3 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="7" t="inlineStr">
@@ -3345,6 +4230,21 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://thedropcomedyclub.com/calendar</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://thedropcomedyclub.com/calendar.html</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Discovered 2 Candidates</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="4" t="inlineStr">
@@ -3375,6 +4275,11 @@
       <c r="F91" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Verified Original</t>
         </is>
       </c>
     </row>

</xml_diff>